<commit_message>
Withdraw marketing shots of the old adult player.
Playable characters are the eight kids, Haruto by default. Screenshots that show the removed adult student or the old character-select models are no longer used on Facebook cards or Word covers. Current plates live in Marketing/HinhAnh/. Posts without a current shot are text cards labeled CẦN ẢNH MỚI.

Co-authored-by: Quách Thành Long  <stephensouth1307@gmail.com>
</commit_message>
<xml_diff>
--- a/Bao_Cao/marketing/Lich_Noi_Dung_12_Tuan.xlsx
+++ b/Bao_Cao/marketing/Lich_Noi_Dung_12_Tuan.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cach dung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lich" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Nam" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cach dung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lich" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nam" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lich'!$A$1:$N$88</definedName>
@@ -875,7 +875,7 @@
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1365,7 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Tuan-02/01-bay-gio-sang/story-1920.png</t>
+          <t>Tuan-02/01-bay-gio-sang/CAN_QUAY.md</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Dùng story khi đã quay lời</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Tuan-04/01-ket-cho-nao/story-1920.png</t>
+          <t>Tuan-04/01-ket-cho-nao/CAN_QUAY.md</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Dùng story khi đã quay lời</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Tuan-05/01-ra-mat-web/story-1920.png</t>
+          <t>Tuan-05/01-ra-mat-web/CAN_QUAY.md</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>Dùng story khi đã quay lời</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4025,7 @@
       </c>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="N55" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="N57" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="N61" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="N63" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -5075,7 +5075,7 @@
       </c>
       <c r="N65" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5285,7 @@
       </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5425,7 @@
       </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Tuan-10/01-an-chay-ngu/story-1920.png</t>
+          <t>Tuan-10/01-an-chay-ngu/CAN_QUAY.md</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="N71" s="5" t="inlineStr">
         <is>
-          <t>Dùng story khi đã quay lời</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="N77" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="N79" s="5" t="inlineStr">
         <is>
-          <t>Sẵn sàng — điền link</t>
+          <t>Cần quay</t>
         </is>
       </c>
     </row>
@@ -9297,7 +9297,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Quyết định dùng horizon_night hay hoãn. Không vẽ bí ngô.</t>
+          <t>Quyết định dùng Marketing/HinhAnh/BoiCanh/pho-dem.jpg hay hoãn. Không vẽ bí ngô.</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Use current kid screenshots on every marketing post.
Play Mode shots of the eight kids already in Bao_Cao replace the placeholder cards. The repo README now leads with those images, the Unity 6000.3.12f1 setup, and only facts checked in the project.

Co-authored-by: Quách Thành Long  <stephensouth1307@gmail.com>
</commit_message>
<xml_diff>
--- a/Bao_Cao/marketing/Lich_Noi_Dung_12_Tuan.xlsx
+++ b/Bao_Cao/marketing/Lich_Noi_Dung_12_Tuan.xlsx
@@ -875,7 +875,7 @@
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1365,7 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Tuan-02/01-bay-gio-sang/CAN_QUAY.md</t>
+          <t>Tuan-02/01-bay-gio-sang/story-1920.png</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Dùng story khi đã quay lời</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Tuan-04/01-ket-cho-nao/CAN_QUAY.md</t>
+          <t>Tuan-04/01-ket-cho-nao/story-1920.png</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Dùng story khi đã quay lời</t>
         </is>
       </c>
     </row>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Tuan-05/01-ra-mat-web/CAN_QUAY.md</t>
+          <t>Tuan-05/01-ra-mat-web/story-1920.png</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Dùng story khi đã quay lời</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="N48" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4025,7 @@
       </c>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="N55" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="N57" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="N61" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="N63" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -5045,7 +5045,7 @@
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>Đảo Midori có nông trại và chỗ câu. Ảnh thật sẽ đăng khi quay xong.</t>
+          <t>Đảo Midori có nông trại và chỗ câu.</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
-          <t>Ảnh sẽ đăng khi quay xong</t>
+          <t>Đảo mở ở 320 trí tuệ với tài khoản</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="N65" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5285,7 @@
       </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5425,7 @@
       </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Tuan-10/01-an-chay-ngu/CAN_QUAY.md</t>
+          <t>Tuan-10/01-an-chay-ngu/story-1920.png</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="N71" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Dùng story khi đã quay lời</t>
         </is>
       </c>
     </row>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="N77" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="N79" s="5" t="inlineStr">
         <is>
-          <t>Cần quay</t>
+          <t>Sẵn sàng — điền link</t>
         </is>
       </c>
     </row>

</xml_diff>